<commit_message>
Update web portal metadata
</commit_message>
<xml_diff>
--- a/meta_data_web_portal/JAX_bulk_RNAseq_release2.xlsx
+++ b/meta_data_web_portal/JAX_bulk_RNAseq_release2.xlsx
@@ -1,739 +1,746 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fredhutch-my.sharepoint.com/personal/byu2_fredhutch_org/Documents/Github/MorPhiC_bulk_RNAseq/meta_data_web_portal/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_E88293383C79E0FDC8A4BA5A779B075C9A1D1A05" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{138A9A3E-2476-D341-A359-E84E68555886}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="1260" yWindow="760" windowWidth="28000" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="238">
-  <si>
-    <t xml:space="preserve">DAV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gene Symbol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRACC Matrix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analysis Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assay Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAV Matrix Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DAV Matrix Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output Image Object</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output Image Location</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plot Title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Script</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fred-Hutch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAFB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq08.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VolcanoPlot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulk RNAseq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_ExM_day_6_MAFB_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq08/processed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExM_day_6_MAFB_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq08/volcano_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExM day 6 MAFB PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step3_check_DE_2025_06_release_JAX_RNAseq08.Rmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DLX3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_DLX3_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_DLX3_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 DLX3 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASCL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_hyp_ASCL2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_hyp_ASCL2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 hyp ASCL2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ELF5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_hyp_ELF5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_hyp_ELF5_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 hyp ELF5 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HIF1A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_hyp_HIF1A_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_hyp_HIF1A_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 hyp HIF1A PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TP63</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_hyp_TP63_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_hyp_TP63_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 hyp TP63 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSX2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_MSX2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_MSX2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 MSX2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_ASCL2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_nor_ASCL2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 nor ASCL2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_ELF5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_nor_ELF5_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 nor ELF5 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_HIF1A_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_nor_HIF1A_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 nor HIF1A PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_TP63_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_nor_TP63_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 nor TP63 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NR2F2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_NR2F2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_NR2F2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 NR2F2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VGLL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_PrS_day_6_nor_VGLL1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_VGLL1_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 VGLL1 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HES5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq09.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_11_HES5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq09/processed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_11_HES5_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq09/volcano_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 11 HES5 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step3_check_DE_2025_06_release_JAX_RNAseq09.Rmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POU3F2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_11_POU3F2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_11_POU3F2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 11 POU3F2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOX1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_11_SOX1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_11_SOX1_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 11 SOX1 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMX2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_14_EMX2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_14_EMX2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 14 EMX2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOXG1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_8_FOXG1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_FOXG1_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 FOXG1 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POU3F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_8_POU3F1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_POU3F1_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 POU3F1 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOX21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_8_SOX21_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_SOX21_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 SOX21 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_CBO_day_9_SP8_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_9_SP8_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 9 SP8 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EOMES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq10.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq10_ENDO_day_5_EOMES_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq10/processed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO_day_5_EOMES_KO.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq10/volcano_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO day 5 EOMES KO vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step3_check_DE_2025_06_release_JAX_RNAseq10.Rmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NKX2-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq10_ENDO_day_5_NKX2-1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO_day_5_NKX2-1_KO.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO day 5 NKX2-1 KO vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq10_MESO_day_5_ISL1_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MESO_day_5_ISL1_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MESO day 5 ISL1 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JAX_RNAseq11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LHX5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v7_JAX_RNAseq3_Prod.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_3_CE_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq11/processed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_CE_LHX5_CE.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq11/volcano_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 CE vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step3_check_DE_2025_06_release_JAX_RNAseq11.Rmd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_3_KO_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_KO_LHX5_KO.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 KO vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_3_PTC_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_PTC_LHX5_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_4_CE_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_CE_LHX5_CE.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 CE vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_4_KO_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_KO_LHX5_KO.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 KO vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_4_PTC_LHX5_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_PTC_LHX5_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FEZF2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_5_CE_FEZF2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_CE_FEZF2_CE.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 CE vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_5_KO_FEZF2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_KO_FEZF2_KO.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 KO vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_CBO_day_5_PTC_FEZF2_DEseq2.tsv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_PTC_FEZF2_PTC.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 PTC vs WT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GOPlot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq08_enrichment.rds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq08/enrichment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_DLX3_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq08/goseq_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 DLX3 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">step4_goseq_2025_06_JAX_RNAseq.sh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_DLX3_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 DLX3 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_ELF5_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 ELF5 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_ELF5_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 ELF5 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_ASCL2_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia ASCL2 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_ASCL2_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia ASCL2 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_ELF5_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia ELF5 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_ELF5_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia ELF5 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_HIF1A_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia HIF1A down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_Hypoxia_HIF1A_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 Hypoxia HIF1A up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_MSX2_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 MSX2 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_MSX2_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 MSX2 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_NR2F2_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 NR2F2 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_NR2F2_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 NR2F2 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS_day_6_VGLL1_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrS day 6 VGLL1 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq09_enrichment.rds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq09/enrichment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_11_SOX1_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq09/goseq_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 11 SOX1 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_14_EMX2_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 14 EMX2 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_POU3F1_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 POU3F1 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_POU3F1_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 POU3F1 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_8_SOX21_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 8 SOX21 up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_9_SP8_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 9 SP8 down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq10_enrichment.rds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq10/enrichment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO_day_5_EOMES_KO_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq10/goseq_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO day 5 EOMES KO down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO_day_5_EOMES_KO_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ENDO day 5 EOMES KO up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025_06_JAX_RNAseq11_enrichment.rds</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq11/enrichment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_CE_LHX5_CE_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq11/goseq_plots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 CE down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_CE_LHX5_CE_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 CE up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_3_LHX5_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 3 LHX5 PTC down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_CE_LHX5_CE_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 CE down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_CE_LHX5_CE_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 CE up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_KO_LHX5_KO_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 KO down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_4_LHX5_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 4 LHX5 PTC down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_CE_FEZF2_CE_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 CE down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_CE_FEZF2_CE_up-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 CE up-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_FEZF2_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 PTC down-regulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO_day_5_KO_FEZF2_KO_down-regulated.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBO day 5 FEZF2 KO down-regulated</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="238">
+  <si>
+    <t>DAV</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Gene Symbol</t>
+  </si>
+  <si>
+    <t>DRACC Matrix</t>
+  </si>
+  <si>
+    <t>Analysis Type</t>
+  </si>
+  <si>
+    <t>Assay Type</t>
+  </si>
+  <si>
+    <t>DAV Matrix Name</t>
+  </si>
+  <si>
+    <t>DAV Matrix Location</t>
+  </si>
+  <si>
+    <t>Output Image Object</t>
+  </si>
+  <si>
+    <t>Output Image Location</t>
+  </si>
+  <si>
+    <t>Plot Title</t>
+  </si>
+  <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>Fred-Hutch</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq08</t>
+  </si>
+  <si>
+    <t>MAFB</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq08.xlsx</t>
+  </si>
+  <si>
+    <t>VolcanoPlot</t>
+  </si>
+  <si>
+    <t>Bulk RNAseq</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_ExM_day_6_MAFB_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq08/processed</t>
+  </si>
+  <si>
+    <t>ExM_day_6_MAFB_PTC.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq08/volcano_plots</t>
+  </si>
+  <si>
+    <t>ExM day 6 MAFB PTC vs WT</t>
+  </si>
+  <si>
+    <t>step3_check_DE_2025_06_release_JAX_RNAseq08.Rmd</t>
+  </si>
+  <si>
+    <t>DLX3</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_DLX3_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_DLX3_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 DLX3 PTC vs WT</t>
+  </si>
+  <si>
+    <t>ASCL2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_hyp_ASCL2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_hyp_ASCL2_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 hyp ASCL2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>ELF5</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_hyp_ELF5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_hyp_ELF5_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 hyp ELF5 PTC vs WT</t>
+  </si>
+  <si>
+    <t>HIF1A</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_hyp_HIF1A_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_hyp_HIF1A_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 hyp HIF1A PTC vs WT</t>
+  </si>
+  <si>
+    <t>TP63</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_hyp_TP63_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_hyp_TP63_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 hyp TP63 PTC vs WT</t>
+  </si>
+  <si>
+    <t>MSX2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_MSX2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_MSX2_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 MSX2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_ASCL2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_nor_ASCL2_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 nor ASCL2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_ELF5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_nor_ELF5_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 nor ELF5 PTC vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_HIF1A_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_nor_HIF1A_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 nor HIF1A PTC vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_TP63_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_nor_TP63_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 nor TP63 PTC vs WT</t>
+  </si>
+  <si>
+    <t>NR2F2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_NR2F2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_NR2F2_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 NR2F2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>VGLL1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_PrS_day_6_nor_VGLL1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>PrS_day_6_VGLL1_PTC.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 VGLL1 PTC vs WT</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq09</t>
+  </si>
+  <si>
+    <t>HES5</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq09.xlsx</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_11_HES5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq09/processed</t>
+  </si>
+  <si>
+    <t>CBO_day_11_HES5_PTC.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq09/volcano_plots</t>
+  </si>
+  <si>
+    <t>CBO day 11 HES5 PTC vs WT</t>
+  </si>
+  <si>
+    <t>step3_check_DE_2025_06_release_JAX_RNAseq09.Rmd</t>
+  </si>
+  <si>
+    <t>POU3F2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_11_POU3F2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_11_POU3F2_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 11 POU3F2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>SOX1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_11_SOX1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_11_SOX1_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 11 SOX1 PTC vs WT</t>
+  </si>
+  <si>
+    <t>EMX2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_14_EMX2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_14_EMX2_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 14 EMX2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>FOXG1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_8_FOXG1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_8_FOXG1_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 FOXG1 PTC vs WT</t>
+  </si>
+  <si>
+    <t>POU3F1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_8_POU3F1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_8_POU3F1_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 POU3F1 PTC vs WT</t>
+  </si>
+  <si>
+    <t>SOX21</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_8_SOX21_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_8_SOX21_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 SOX21 PTC vs WT</t>
+  </si>
+  <si>
+    <t>SP8</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_CBO_day_9_SP8_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_9_SP8_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 9 SP8 PTC vs WT</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq10</t>
+  </si>
+  <si>
+    <t>EOMES</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq10.xlsx</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq10_ENDO_day_5_EOMES_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq10/processed</t>
+  </si>
+  <si>
+    <t>ENDO_day_5_EOMES_KO.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq10/volcano_plots</t>
+  </si>
+  <si>
+    <t>ENDO day 5 EOMES KO vs WT</t>
+  </si>
+  <si>
+    <t>step3_check_DE_2025_06_release_JAX_RNAseq10.Rmd</t>
+  </si>
+  <si>
+    <t>NKX2-1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq10_ENDO_day_5_NKX2-1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>ENDO_day_5_NKX2-1_KO.png</t>
+  </si>
+  <si>
+    <t>ENDO day 5 NKX2-1 KO vs WT</t>
+  </si>
+  <si>
+    <t>ISL1</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq10_MESO_day_5_ISL1_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>MESO_day_5_ISL1_PTC.png</t>
+  </si>
+  <si>
+    <t>MESO day 5 ISL1 PTC vs WT</t>
+  </si>
+  <si>
+    <t>JAX_RNAseq_Neuroectoderm</t>
+  </si>
+  <si>
+    <t>LHX5</t>
+  </si>
+  <si>
+    <t>v7_JAX_RNAseq3_Prod.xlsx</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_3_CE_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq11/processed</t>
+  </si>
+  <si>
+    <t>CBO_day_3_CE_LHX5_CE.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq11/volcano_plots</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 CE vs WT</t>
+  </si>
+  <si>
+    <t>step3_check_DE_2025_06_release_JAX_RNAseq11.Rmd</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_3_KO_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_3_KO_LHX5_KO.png</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 KO vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_3_PTC_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_3_PTC_LHX5_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 PTC vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_4_CE_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_4_CE_LHX5_CE.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 CE vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_4_KO_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_4_KO_LHX5_KO.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 KO vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_4_PTC_LHX5_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_4_PTC_LHX5_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 PTC vs WT</t>
+  </si>
+  <si>
+    <t>FEZF2</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_5_CE_FEZF2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_5_CE_FEZF2_CE.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 CE vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_5_KO_FEZF2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_5_KO_FEZF2_KO.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 KO vs WT</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_CBO_day_5_PTC_FEZF2_DEseq2.tsv</t>
+  </si>
+  <si>
+    <t>CBO_day_5_PTC_FEZF2_PTC.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 PTC vs WT</t>
+  </si>
+  <si>
+    <t>GOPlot</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq08_enrichment.rds</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq08/enrichment</t>
+  </si>
+  <si>
+    <t>PrS_day_6_DLX3_down-regulated.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq08/goseq_plots</t>
+  </si>
+  <si>
+    <t>PrS day 6 DLX3 down-regulated</t>
+  </si>
+  <si>
+    <t>step4_goseq_2025_06_JAX_RNAseq.sh</t>
+  </si>
+  <si>
+    <t>PrS_day_6_DLX3_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 DLX3 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_ELF5_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 ELF5 down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_ELF5_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 ELF5 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_ASCL2_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia ASCL2 down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_ASCL2_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia ASCL2 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_ELF5_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia ELF5 down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_ELF5_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia ELF5 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_HIF1A_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia HIF1A down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_Hypoxia_HIF1A_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 Hypoxia HIF1A up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_MSX2_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 MSX2 down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_MSX2_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 MSX2 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_NR2F2_down-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 NR2F2 down-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_NR2F2_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 NR2F2 up-regulated</t>
+  </si>
+  <si>
+    <t>PrS_day_6_VGLL1_up-regulated.png</t>
+  </si>
+  <si>
+    <t>PrS day 6 VGLL1 up-regulated</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq09_enrichment.rds</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq09/enrichment</t>
+  </si>
+  <si>
+    <t>CBO_day_11_SOX1_up-regulated.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq09/goseq_plots</t>
+  </si>
+  <si>
+    <t>CBO day 11 SOX1 up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_14_EMX2_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 14 EMX2 down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_8_POU3F1_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 POU3F1 down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_8_POU3F1_up-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 POU3F1 up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_8_SOX21_up-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 8 SOX21 up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_9_SP8_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 9 SP8 down-regulated</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq10_enrichment.rds</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq10/enrichment</t>
+  </si>
+  <si>
+    <t>ENDO_day_5_EOMES_KO_down-regulated.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq10/goseq_plots</t>
+  </si>
+  <si>
+    <t>ENDO day 5 EOMES KO down-regulated</t>
+  </si>
+  <si>
+    <t>ENDO_day_5_EOMES_KO_up-regulated.png</t>
+  </si>
+  <si>
+    <t>ENDO day 5 EOMES KO up-regulated</t>
+  </si>
+  <si>
+    <t>2025_06_JAX_RNAseq11_enrichment.rds</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/results/2025_06_JAX_RNAseq11/enrichment</t>
+  </si>
+  <si>
+    <t>CBO_day_3_CE_LHX5_CE_down-regulated.png</t>
+  </si>
+  <si>
+    <t>MorPhiC_bulk_RNAseq/figures/2025_06_JAX_RNAseq11/goseq_plots</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 CE down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_3_CE_LHX5_CE_up-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 CE up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_3_LHX5_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 3 LHX5 PTC down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_4_CE_LHX5_CE_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 CE down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_4_CE_LHX5_CE_up-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 CE up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_4_KO_LHX5_KO_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 KO down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_4_LHX5_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 4 LHX5 PTC down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_5_CE_FEZF2_CE_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 CE down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_5_CE_FEZF2_CE_up-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 CE up-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_5_FEZF2_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 PTC down-regulated</t>
+  </si>
+  <si>
+    <t>CBO_day_5_KO_FEZF2_KO_down-regulated.png</t>
+  </si>
+  <si>
+    <t>CBO day 5 FEZF2 KO down-regulated</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -769,6 +776,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1050,11 +1066,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L68"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="47.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1092,7 +1112,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1130,7 +1150,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1168,7 +1188,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1206,7 +1226,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1244,7 +1264,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1282,7 +1302,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1320,7 +1340,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1358,7 +1378,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1396,7 +1416,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1434,7 +1454,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1472,7 +1492,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1510,7 +1530,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1548,7 +1568,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1586,7 +1606,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1624,7 +1644,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
@@ -1662,7 +1682,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>12</v>
       </c>
@@ -1700,7 +1720,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -1738,7 +1758,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -1776,7 +1796,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1814,7 +1834,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -1852,7 +1872,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1890,7 +1910,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1928,7 +1948,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -1966,7 +1986,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -2004,7 +2024,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
@@ -2042,7 +2062,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -2080,7 +2100,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -2118,7 +2138,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -2156,7 +2176,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>12</v>
       </c>
@@ -2194,7 +2214,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -2232,7 +2252,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -2270,7 +2290,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -2308,7 +2328,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -2346,7 +2366,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -2384,7 +2404,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>12</v>
       </c>
@@ -2422,7 +2442,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -2460,7 +2480,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -2498,7 +2518,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>12</v>
       </c>
@@ -2536,7 +2556,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>12</v>
       </c>
@@ -2574,7 +2594,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>12</v>
       </c>
@@ -2612,7 +2632,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>12</v>
       </c>
@@ -2650,7 +2670,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>12</v>
       </c>
@@ -2688,7 +2708,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>12</v>
       </c>
@@ -2726,7 +2746,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>12</v>
       </c>
@@ -2764,7 +2784,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>12</v>
       </c>
@@ -2802,7 +2822,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>12</v>
       </c>
@@ -2840,7 +2860,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>12</v>
       </c>
@@ -2878,7 +2898,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>12</v>
       </c>
@@ -2916,7 +2936,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>12</v>
       </c>
@@ -2954,7 +2974,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>12</v>
       </c>
@@ -2992,7 +3012,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -3030,7 +3050,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>12</v>
       </c>
@@ -3068,7 +3088,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>12</v>
       </c>
@@ -3106,7 +3126,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>12</v>
       </c>
@@ -3144,7 +3164,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>12</v>
       </c>
@@ -3182,7 +3202,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>12</v>
       </c>
@@ -3220,7 +3240,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>12</v>
       </c>
@@ -3258,7 +3278,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>12</v>
       </c>
@@ -3296,7 +3316,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>12</v>
       </c>
@@ -3334,7 +3354,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>12</v>
       </c>
@@ -3372,7 +3392,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>12</v>
       </c>
@@ -3410,7 +3430,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>12</v>
       </c>
@@ -3448,7 +3468,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>12</v>
       </c>
@@ -3486,7 +3506,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>12</v>
       </c>
@@ -3524,7 +3544,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>12</v>
       </c>
@@ -3562,7 +3582,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -3600,7 +3620,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>12</v>
       </c>
@@ -3640,6 +3660,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>